<commit_message>
Prepare GovTribe 1.2.0 for directory review
</commit_message>
<xml_diff>
--- a/skills/govtribe-file-templates/assets/proposal-control-workbook/proposal-control-workbook.xlsx
+++ b/skills/govtribe-file-templates/assets/proposal-control-workbook/proposal-control-workbook.xlsx
@@ -69,7 +69,7 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
-    <author>GovTribe</author>
+    <author>OpenAI</author>
   </authors>
   <commentList>
     <comment ref="B5" authorId="0">
@@ -175,7 +175,7 @@
 <file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
-    <author>GovTribe</author>
+    <author>OpenAI</author>
   </authors>
   <commentList>
     <comment ref="E7" authorId="0">
@@ -293,7 +293,7 @@
 <file path=xl/comments5.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
-    <author>GovTribe</author>
+    <author>OpenAI</author>
   </authors>
   <commentList>
     <comment ref="B7" authorId="0">

</xml_diff>